<commit_message>
Squashed commit of the following:
commit f2943a6bc33a96f4b66774e600ca332be452f052
Author: kmj710100-lang <kmj710100@gmail.com>
Date:   Fri Oct 23 15:18:44 2026 +0900

    10/23 기획서 수정

    Zomso_Parrying_기획서.docx
    1.1 기획 의도 내용 수정 (적 오브젝트의 패링 범주 설명)

    SBSAcademy_Team01_기획서.docx
    1 기획의도 내용 전면 수정.
    3.5 스테이지 전개 시스템 목차 제거.

commit b3e2969d8b5b59026a7daef9c29ef3559179c3c8
Author: kmj710100-lang <kmj710100@gmail.com>
Date:   Fri Oct 23 01:57:52 2026 +0900

    10/23_0 기획서 및 UI 배치 수정 및 작성

    SBSAcademy_Team01_기획서.docx
    3.3.2 약공격 스킬 내용 수정 .(쿨타임 시스템 제거)
    4.2 몬스터 HPbar 협의 필요로 내용 전환.
    4.3 보스 그로기 타임 관련 내용 추가.

    씬 별 UI.pptx
    플레이 씬 UI 배치 수정 (좌측 4버튼 / 우측 레버 및 1버튼)

    Zomso_Parrying_기획서.docx
    패링 관련 세부 기획서 작성
</commit_message>
<xml_diff>
--- a/SkillDatatable.xlsx
+++ b/SkillDatatable.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="현재_통합_문서" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1119,7 +1119,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1163,9 +1163,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1522,7 +1519,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42A07B8D-296F-4731-B27A-9CC1CD5CA71B}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AH15"/>
+  <dimension ref="A1:AH13"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.625" style="1" bestFit="1" customWidth="1"/>
@@ -2067,10 +2064,10 @@
       <c r="C13" s="1">
         <v>10011</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="1" t="s">
         <v>128</v>
       </c>
       <c r="F13" s="1" t="s">
@@ -2085,14 +2082,6 @@
       <c r="J13" s="1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-    </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.3">
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>